<commit_message>
Fixed missing Int sum column
</commit_message>
<xml_diff>
--- a/UO_Suit_Builder.xlsx
+++ b/UO_Suit_Builder.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="P:\Documents\Ultima Online\UltimaOnline_Suit-Builder\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3BFED56E-B098-4285-9704-4706A7040758}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{65F73BEB-55DD-4663-BEC2-56A6E837928C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="48660" yWindow="2304" windowWidth="38268" windowHeight="21360" xr2:uid="{A0B388F1-62EB-4C63-B127-49B54EA8858F}"/>
+    <workbookView xWindow="47340" yWindow="1740" windowWidth="38268" windowHeight="21000" xr2:uid="{A0B388F1-62EB-4C63-B127-49B54EA8858F}"/>
   </bookViews>
   <sheets>
     <sheet name="Suit Template" sheetId="13" r:id="rId1"/>
@@ -2553,7 +2553,10 @@
         <f>SUM(H20:H21)</f>
         <v>0</v>
       </c>
-      <c r="I22" s="20"/>
+      <c r="I22" s="20">
+        <f>SUM(I20:I21)</f>
+        <v>0</v>
+      </c>
       <c r="J22" s="19">
         <f>IF(J20&gt;=25,G22/2+75,G22/2+50+J20)</f>
         <v>50</v>
@@ -3068,6 +3071,27 @@
     </row>
   </sheetData>
   <mergeCells count="30">
+    <mergeCell ref="C22:D22"/>
+    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="N22:O22"/>
+    <mergeCell ref="P22:Q22"/>
+    <mergeCell ref="A1:A2"/>
+    <mergeCell ref="B1:F1"/>
+    <mergeCell ref="G1:L1"/>
+    <mergeCell ref="M1:O1"/>
+    <mergeCell ref="P1:U1"/>
+    <mergeCell ref="AC1:AE1"/>
+    <mergeCell ref="AG1:AL1"/>
+    <mergeCell ref="C21:D21"/>
+    <mergeCell ref="E21:F21"/>
+    <mergeCell ref="J21:L21"/>
+    <mergeCell ref="V1:AB1"/>
+    <mergeCell ref="N24:O24"/>
+    <mergeCell ref="P24:Q24"/>
+    <mergeCell ref="C25:E26"/>
+    <mergeCell ref="F25:F26"/>
+    <mergeCell ref="G25:G26"/>
+    <mergeCell ref="H25:H26"/>
     <mergeCell ref="C33:E33"/>
     <mergeCell ref="C34:E34"/>
     <mergeCell ref="C35:E35"/>
@@ -3077,27 +3101,6 @@
     <mergeCell ref="C30:E30"/>
     <mergeCell ref="C31:E31"/>
     <mergeCell ref="C32:E32"/>
-    <mergeCell ref="N24:O24"/>
-    <mergeCell ref="P24:Q24"/>
-    <mergeCell ref="C25:E26"/>
-    <mergeCell ref="F25:F26"/>
-    <mergeCell ref="G25:G26"/>
-    <mergeCell ref="H25:H26"/>
-    <mergeCell ref="AC1:AE1"/>
-    <mergeCell ref="AG1:AL1"/>
-    <mergeCell ref="C21:D21"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="J21:L21"/>
-    <mergeCell ref="V1:AB1"/>
-    <mergeCell ref="C22:D22"/>
-    <mergeCell ref="E22:F22"/>
-    <mergeCell ref="N22:O22"/>
-    <mergeCell ref="P22:Q22"/>
-    <mergeCell ref="A1:A2"/>
-    <mergeCell ref="B1:F1"/>
-    <mergeCell ref="G1:L1"/>
-    <mergeCell ref="M1:O1"/>
-    <mergeCell ref="P1:U1"/>
   </mergeCells>
   <conditionalFormatting sqref="J20">
     <cfRule type="cellIs" dxfId="11" priority="12" operator="greaterThan">

</xml_diff>